<commit_message>
feat: add driver3 field to support 3-driver entries for R1
</commit_message>
<xml_diff>
--- a/public/templates/inje-gt-masters_results_template.xlsx
+++ b/public/templates/inje-gt-masters_results_template.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -531,13 +531,14 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -568,35 +569,40 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>드라이버3</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>차량</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>랩수</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>총시간</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>갭</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>패스티스트</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>포인트</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
@@ -618,37 +624,38 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>홍길동</t>
+          <t>김태환</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>김철수</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+          <t>이인용</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>아반떼 N</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>0:45:12.345</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>1:45.678</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="L2" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>classified</t>
         </is>
@@ -660,47 +667,56 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>레이싱랩</t>
+          <t>AXIS Racing</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>이영희</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
+          <t>이운영</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>홍준기</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>조예찬</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>벨로스터 N</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>0:45:18.901</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>+6.556</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>1:46.123</t>
         </is>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="L3" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>classified</t>
         </is>
@@ -730,29 +746,30 @@
           <t>정수연</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>아반떼 N</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>+2 laps</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>1:47.890</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="L4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>dnf</t>
         </is>
@@ -767,7 +784,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A5:M5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -779,7 +796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -954,7 +971,7 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>차량</t>
+          <t>드라이버3</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -969,19 +986,19 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>차량 모델명</t>
+          <t>공동 드라이버 3번째. 3인 참가 시 입력</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>아반떼 N</t>
+          <t>박재현</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>랩수</t>
+          <t>차량</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -991,24 +1008,24 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>완주한 랩 수</t>
+          <t>차량 모델명</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>아반떼 N</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>총시간</t>
+          <t>랩수</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1018,24 +1035,24 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>시:분:초.밀리</t>
+          <t>정수</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>완주 총 시간. DNF/DNS/DSQ는 공란</t>
+          <t>완주한 랩 수</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>0:45:12.345</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>갭</t>
+          <t>총시간</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -1045,24 +1062,24 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>텍스트</t>
+          <t>시:분:초.밀리</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>선두와의 차이. 1위는 공란, 랩차는 '+N laps'</t>
+          <t>완주 총 시간. DNF/DNS/DSQ는 공란</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>+6.556, +2 laps</t>
+          <t>0:45:12.345</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>패스티스트</t>
+          <t>갭</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1072,24 +1089,24 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>분:초.밀리</t>
+          <t>텍스트</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>최고 랩 타임</t>
+          <t>선두와의 차이. 1위는 공란, 랩차는 '+N laps'</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>1:45.678</t>
+          <t>+6.556, +2 laps</t>
         </is>
       </c>
     </row>
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>포인트</t>
+          <t>패스티스트</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -1099,42 +1116,69 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>분:초.밀리</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>획득 포인트. 0도 명시 권장</t>
+          <t>최고 랩 타임</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>25, 18, 15</t>
+          <t>1:45.678</t>
         </is>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>포인트</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>선택</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>정수</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>획득 포인트. 0도 명시 권장</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>25, 18, 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>영문 소문자 4가지 중 하나</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>classified=완주 / dnf=Did Not Finish / dns=Did Not Start / dsq=Disqualified. 생략 시 classified</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>classified</t>
         </is>

</xml_diff>